<commit_message>
Replace Raw Milk Production data with Casey's weekly KPI log, add CWT column, correct Annual Production and monthly chart
</commit_message>
<xml_diff>
--- a/data/Raw Milk Production - Stat Cards.xlsx
+++ b/data/Raw Milk Production - Stat Cards.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8160" yWindow="4340" windowWidth="22080" windowHeight="14160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,7 +25,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -54,7 +56,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -418,14 +420,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="3" max="4"/>
+    <col width="20" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,22 +441,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TTM Jul 2026</t>
+          <t>Average TTM Jul 2026</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TTM Jul 2025</t>
+          <t>Average TTM Jul 2025</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>TTM Jul 2026 (gal)</t>
+          <t>Average TTM Jul 2026 (gal)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TTM Jul 2025 (gal)</t>
+          <t>Average TTM Jul 2025 (gal)</t>
         </is>
       </c>
     </row>
@@ -471,13 +471,17 @@
           <t>hundredweight (cwt)</t>
         </is>
       </c>
-      <c r="E2">
-        <f>C2*11.63</f>
-        <v/>
-      </c>
-      <c r="F2">
-        <f>D2*11.63</f>
-        <v/>
+      <c r="C2" t="n">
+        <v>40991.46</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40844.88</v>
+      </c>
+      <c r="E2" t="n">
+        <v>476731</v>
+      </c>
+      <c r="F2" t="n">
+        <v>475026</v>
       </c>
     </row>
     <row r="3">
@@ -490,6 +494,14 @@
         <is>
           <t>vs. MI state avg</t>
         </is>
+      </c>
+      <c r="E3">
+        <f>8.6*E2</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>8.6*F2</f>
+        <v/>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Fix Raw Milk Production units: KPI sheet's Actual column is gallons, not pounds; recompute Annual Production, monthly chart, and CWT column
</commit_message>
<xml_diff>
--- a/data/Raw Milk Production - Stat Cards.xlsx
+++ b/data/Raw Milk Production - Stat Cards.xlsx
@@ -472,16 +472,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40991.46</v>
+        <v>352526.51</v>
       </c>
       <c r="D2" t="n">
-        <v>40844.88</v>
+        <v>351266</v>
       </c>
       <c r="E2" t="n">
-        <v>476731</v>
+        <v>4099146</v>
       </c>
       <c r="F2" t="n">
-        <v>475026</v>
+        <v>4084488</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Fill Lbs/Cow/Day stat card, reorder Monthly Production chart to fiscal Jul-Jun axis
</commit_message>
<xml_diff>
--- a/data/Raw Milk Production - Stat Cards.xlsx
+++ b/data/Raw Milk Production - Stat Cards.xlsx
@@ -492,8 +492,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>vs. MI state avg</t>
-        </is>
+          <t>vs. MI state avg (76.7), last 4 weeks avg</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>83.59999999999999</v>
       </c>
       <c r="E3">
         <f>8.6*E2</f>

</xml_diff>